<commit_message>
Aggiunto es di TPSI e modifica dei file excel di GPOI
</commit_message>
<xml_diff>
--- a/5°anno/GPOI/es_pag6(c).xlsx
+++ b/5°anno/GPOI/es_pag6(c).xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25128"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\crist\Desktop\FILE SCUOLA\Cartella Repository\repository_generale\5°anno\GPOI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\crist\Desktop\repository_generale\5°anno\GPOI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5772FBB-1890-4324-A992-012E7401C2FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4279583-CC0B-4AA9-9EDB-502054B3F153}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B2A40651-5BF7-439F-A35A-CFCF6A0A3041}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -23,12 +23,8 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -39,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
   <si>
     <t>prezzo</t>
   </si>
@@ -85,12 +81,15 @@
   <si>
     <t>p = - (3/10)q + 24</t>
   </si>
+  <si>
+    <t>p * q = 3 * 70 = 210</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -625,7 +624,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -633,6 +631,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1582,17 +1581,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3532729-CEDF-491A-A710-414283DF0114}">
   <dimension ref="A1:J18"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="4" max="4" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.21875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.09765625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.59765625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.8984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.3984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.19921875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.796875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1602,8 +1602,11 @@
       <c r="D1" t="s">
         <v>2</v>
       </c>
+      <c r="E1" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10">
       <c r="A2">
         <f xml:space="preserve"> 24 - (3 / 10) * B2</f>
         <v>24</v>
@@ -1618,7 +1621,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10">
       <c r="A3">
         <f t="shared" ref="A3:A18" si="0" xml:space="preserve"> 24 - (3 / 10) * B3</f>
         <v>22.5</v>
@@ -1642,7 +1645,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10">
       <c r="A4">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -1669,7 +1672,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>19.5</v>
@@ -1678,7 +1681,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -1687,7 +1690,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10">
       <c r="A7">
         <f t="shared" si="0"/>
         <v>16.5</v>
@@ -1696,7 +1699,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10">
       <c r="A8">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1705,7 +1708,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10">
       <c r="A9">
         <f t="shared" si="0"/>
         <v>13.5</v>
@@ -1714,7 +1717,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10">
       <c r="A10">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1723,7 +1726,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10">
       <c r="A11">
         <f t="shared" si="0"/>
         <v>10.5</v>
@@ -1732,7 +1735,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10">
       <c r="A12">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1741,7 +1744,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10">
       <c r="A13">
         <f t="shared" si="0"/>
         <v>7.5</v>
@@ -1750,7 +1753,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10">
       <c r="A14">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1759,7 +1762,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10">
       <c r="A15">
         <f t="shared" si="0"/>
         <v>4.5</v>
@@ -1768,7 +1771,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10">
       <c r="A16">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -1777,7 +1780,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2">
       <c r="A17">
         <f t="shared" si="0"/>
         <v>1.5</v>
@@ -1786,7 +1789,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2">
       <c r="A18">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1797,6 +1800,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>